<commit_message>
Issue #1/#5: enriquecer el corpus y consistencia de citas
Documentos (más planes y detalle):
- comparativa_planes.csv: nuevo plan Starter + ~27 características comparadas.
- planes_y_precios.xlsx: hojas Planes, Add-ons, Descuentos y Detalle por plan.
- base_conocimiento.md: sección de planes, seguridad, reportes, móvil, más detalle.
- integraciones_api.json: más endpoints, integraciones, webhooks y códigos de error.
- faq_soporte.html: muchas más FAQ (reembolsos, descuentos, datos, idiomas...).
- onboarding_producto.pptx, terminos_de_uso.docx, politica_privacidad.pdf ampliados.

Generación:
- _remap_citations: renumera los [n] del texto para que coincidan exactamente con
  la lista de fuentes citadas y deduplica por archivo (reemplaza a _cited_sources).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/documents/comercial/planes_y_precios.xlsx
+++ b/data/documents/comercial/planes_y_precios.xlsx
@@ -9,6 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Planes y Precios" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Add-ons" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Descuentos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detalle por plan" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -435,6 +437,31 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>Ahorro anual</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Usuarios incluidos</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Almacenamiento</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Soporte</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>SLA uptime</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>Público objetivo</t>
         </is>
       </c>
@@ -453,63 +480,206 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Equipos pequeños que inician</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1 GB</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Comunidad</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Equipos que inician</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Pro</t>
+          <t>Starter</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C3" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Equipos en crecimiento</t>
+          <t>17%</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>10 GB</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Email (72 h)</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>99.0%</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Equipos pequeños</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Pro</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="C4" t="n">
-        <v>180</v>
+        <v>90</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Empresas con varios equipos</t>
+          <t>17%</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Ilimitado</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>50 GB</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Email (48 h)</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>99.5%</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Equipos en crecimiento</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>18</v>
+      </c>
+      <c r="C5" t="n">
+        <v>180</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>17%</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Ilimitado</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>200 GB</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Email + Chat (8 h)</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>99.9%</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Empresas con varios equipos</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>Enterprise</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Personalizado</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Personalizado</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Negociable</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Ilimitado</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Ilimitado</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Dedicado 24/7 (1 h SLA)</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>99.95%</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
         <is>
           <t>Grandes organizaciones</t>
         </is>
@@ -526,7 +696,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -587,7 +757,271 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Inicio de sesión único corporativo</t>
+          <t>Inicio de sesión único corporativo (incluido en Enterprise)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Automatizaciones extra (+5000/mes)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>29</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Más ejecuciones de reglas por mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Sandbox de pruebas</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>39</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Entorno aislado para probar configuraciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Retención de auditoría extendida</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>59</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Conserva registros de auditoría por más tiempo</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Condición</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Pago anual</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>17%</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Se pagan 10 meses por año</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Instituciones educativas verificadas</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ONG / Sin fines de lucro</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Organizaciones verificadas</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Volumen 50+ usuarios</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>A partir de 50 licencias</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Volumen 200+ usuarios</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>A partir de 200 licencias</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Startups</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>25% primer año</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Programa TechNova for Startups</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Detalle</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Hasta 5 usuarios, 3 proyectos, 1 GB y vistas Kanban/Lista. Ideal para probar la plataforma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Starter</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Hasta 15 usuarios, 20 proyectos, 10 GB, vista Calendario, invitados externos y soporte por email.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Usuarios ilimitados, 50 GB, vista Gantt, acceso a la API (1000/h) y todas las integraciones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>200 GB, roles personalizados, reportes avanzados, registros de auditoría (90 días) y soporte por email + chat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Enterprise</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Almacenamiento ilimitado, SSO/SAML incluido, SLA 99.95%, soporte dedicado 24/7 y CSM asignado.</t>
         </is>
       </c>
     </row>

</xml_diff>